<commit_message>
21-4140 updated excel file
</commit_message>
<xml_diff>
--- a/teams/benefits-portfolio/benefits-intake-optimization-pingwind/post-go-live/21-4140/21-4140-post-go-live-submission-tracker.xlsx
+++ b/teams/benefits-portfolio/benefits-intake-optimization-pingwind/post-go-live/21-4140/21-4140-post-go-live-submission-tracker.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="63">
   <si>
     <t xml:space="preserve">21-4140 Post-Go-Live Submission Tracker</t>
   </si>
@@ -194,6 +194,21 @@
   </si>
   <si>
     <t xml:space="preserve">31033a9b-fbe5-41ab-bdf3-4ce3cde56d6a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7fb98236-eafa-40fe-8d87-9ec444603061</t>
+  </si>
+  <si>
+    <t xml:space="preserve">724eb0f9-5854-4982-b770-8c2af055f7bd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4550c7bf-51b7-4573-ac58-20be3d90fb75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c1745883-9d3a-48b5-95fe-00af5fc5e845</t>
+  </si>
+  <si>
+    <t xml:space="preserve">add33c14-32f7-4e2a-a970-25348707bfe5</t>
   </si>
 </sst>
 </file>
@@ -630,11 +645,11 @@
       </c>
       <c r="B4" s="1" t="n">
         <f aca="false">COUNTIF(A11:A70,"*")-COUNT(A11:A70)</f>
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C4" s="6" t="n">
         <f aca="false">B4/B3</f>
-        <v>0.0102442868400315</v>
+        <v>0.0115576569477279</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1471,37 +1486,81 @@
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="10"/>
-      <c r="B50" s="11"/>
-      <c r="C50" s="13"/>
-      <c r="D50" s="11"/>
-      <c r="E50" s="13"/>
+      <c r="A50" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B50" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C50" s="13" t="n">
+        <v>46087.4659722222</v>
+      </c>
+      <c r="D50" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E50" s="13" t="n">
+        <v>46087.6770833333</v>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>69666796</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="10"/>
-      <c r="B51" s="11"/>
-      <c r="C51" s="13"/>
-      <c r="D51" s="11"/>
-      <c r="E51" s="13"/>
+      <c r="A51" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B51" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C51" s="13" t="n">
+        <v>46087.9388888889</v>
+      </c>
+      <c r="D51" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E51" s="13" t="n">
+        <v>46088.4194444444</v>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>69691895</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="10"/>
-      <c r="B52" s="11"/>
-      <c r="C52" s="13"/>
+      <c r="A52" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B52" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C52" s="13" t="n">
+        <v>46090.8319444444</v>
+      </c>
       <c r="D52" s="11"/>
       <c r="E52" s="13"/>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="10"/>
-      <c r="B53" s="11"/>
-      <c r="C53" s="13"/>
+      <c r="A53" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B53" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C53" s="13" t="n">
+        <v>46090.9305555556</v>
+      </c>
       <c r="D53" s="11"/>
       <c r="E53" s="13"/>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="10"/>
-      <c r="B54" s="11"/>
-      <c r="C54" s="13"/>
+      <c r="A54" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="B54" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C54" s="13" t="n">
+        <v>46091.4236111111</v>
+      </c>
       <c r="D54" s="11"/>
       <c r="E54" s="13"/>
     </row>

</xml_diff>

<commit_message>
Update post-go-live tracking for 21-8940 and 21-4140
</commit_message>
<xml_diff>
--- a/teams/benefits-portfolio/benefits-intake-optimization-pingwind/post-go-live/21-4140/21-4140-post-go-live-submission-tracker.xlsx
+++ b/teams/benefits-portfolio/benefits-intake-optimization-pingwind/post-go-live/21-4140/21-4140-post-go-live-submission-tracker.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="162">
   <si>
     <t xml:space="preserve">21-4140 Post-Go-Live Submission Tracker</t>
   </si>
@@ -209,6 +209,303 @@
   </si>
   <si>
     <t xml:space="preserve">add33c14-32f7-4e2a-a970-25348707bfe5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5c3b51e7-0ecc-4523-9c9e-ee4480a8af88</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Success</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/12/2026 10:46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fc528242-5eca-499a-af53-08bbef6d190b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/12/2026 10:52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c69aa806-f001-4c11-8410-d92703eabfb1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/12/2026 19:11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5da48501-f708-4dcb-835c-6e0bda4aa140</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/13/2026 09:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c23fb21f-3ae9-49f4-baa8-73b544916ca8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/15/2026 21:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">563f9b82-d493-4b75-9ca6-cbd7cde54cb4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/16/2026 17:09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">af362230-1f14-47b4-99bd-aef6bfaf0908</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/16/2026 17:11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31958767-b377-4e47-bce5-582ce4e0daf9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/16/2026 20:26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">80429ad7-605b-44e1-9c3c-e4476c93cf7f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/18/2026 13:32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e6297774-131c-4fad-beae-42bc1f763208</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/18/2026 13:37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26054207-5940-4658-a4c6-f5905ed60f1d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/18/2026 14:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6937e0ff-11ce-4871-8e1f-fea0481abc8e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/18/2026 15:09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7d27d9ba-40df-449e-b648-9ca84bd2e5ad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/19/2026 22:32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9a007d47-e752-41c3-858e-3e0f3a25d2a4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/20/2026 12:32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15ea917a-cca9-414d-a7e5-06945b40c68c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/20/2026 20:55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5d2df05b-36fb-44e8-8195-fadd2c48b859</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/23/2026 07:37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bf2c4d11-bfd6-431e-9fa1-9cc81e4ffe5f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/23/2026 10:59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d829f8ad-055b-4dca-a5e8-3aac12a01ff8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/24/2026 01:14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3d7a0d9b-4743-4af3-9a92-50b82e9837a9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/24/2026 14:14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fb54d4a6-e6b4-4818-aae2-04e99dccf8ce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/25/2026 08:27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8d929786-87d7-4351-818c-482fdb0559f2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/25/2026 10:24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a727ea0c-f323-435d-8700-9e2bddba8fb6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/26/2026 13:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3a8b5ee6-c30e-4622-9ca9-248f78d20546</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/26/2026 18:45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d35c90c0-489e-4873-abce-c85961170979</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/26/2026 19:37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">90d8293d-915e-4db2-9872-b184853f0b39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/26/2026 20:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2fe104bc-bc1b-4463-bbc5-0af5f49ba8f1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/26/2026 22:48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24b3ebc7-489a-4451-b5af-02fa595cc584</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/27/2026 08:54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b9d11296-72fb-4fc4-80eb-b8e6885773ed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/27/2026 14:34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">704b5e6a-1953-4c74-bd6d-392e0f5093f6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/27/2026 19:10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26a4f23d-94b9-4194-b864-aa884a027574</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/28/2026 01:53</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5e22bf60-b82f-47bc-92a4-091d556d9dd5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/28/2026 10:49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d2e4adab-bbde-4d68-9320-f60c5072c194</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/28/2026 20:28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a95d817f-80bc-4d76-bad7-714adf8f9b93</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/29/2026 06:57</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6ff9696e-4b29-462e-99f6-d0373143e945</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/29/2026 18:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5591c8cf-0399-44a9-8efa-2bd9536b97c2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/30/2026 05:20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">76bebd21-5dfe-44b3-99ce-6ffcceb6ccb8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/30/2026 10:42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2570e4df-7a2b-4677-be74-2895137445c0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/30/2026 11:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">589b3dc5-f296-448a-9430-ab48d0428913</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/30/2026 12:18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b6570d1a-4401-47e5-9387-b78e44c992c9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/30/2026 18:44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aa1d974b-9e45-44fb-8b85-9905b25b44c3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/30/2026 21:18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">697e2deb-3207-4444-99e8-5f8d52baf28a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/31/2026 07:47</t>
+  </si>
+  <si>
+    <t xml:space="preserve">89968a27-b320-4c65-93fe-293aa3e851b9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/31/2026 14:05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6f7274a2-5a07-49b4-aca6-86c98edd8c53</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/31/2026 16:02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5425c3b4-c4d2-417d-84d3-e99cefdcdeb3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04/01/2026 09:48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9121103f-ef2e-4fcf-a827-e28ca388c475</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04/02/2026 17:34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2ec7c563-a71d-4f6d-81f2-a2bd930be182</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04/03/2026 14:02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">327f7b82-2265-4fe8-b774-fd092b52f9b9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04/04/2026 05:07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">49b389bc-cef5-4979-b4f1-7ef98b6c38a2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04/05/2026 12:22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e1132c43-a626-4f78-a569-69615fd10b54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04/05/2026 23:05</t>
   </si>
 </sst>
 </file>
@@ -644,12 +941,12 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="n">
-        <f aca="false">COUNTIF(A11:A70,"*")-COUNT(A11:A70)</f>
-        <v>44</v>
+        <f aca="false">COUNTIF(A11:A270,"*")-COUNT(A11:A270)</f>
+        <v>93</v>
       </c>
       <c r="C4" s="6" t="n">
         <f aca="false">B4/B3</f>
-        <v>0.0115576569477279</v>
+        <v>0.0244286840031521</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1565,1846 +1862,2429 @@
       <c r="E54" s="13"/>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="10"/>
-      <c r="B55" s="11"/>
-      <c r="C55" s="13"/>
+      <c r="A55" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B55" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C55" s="13" t="s">
+        <v>65</v>
+      </c>
       <c r="D55" s="11"/>
       <c r="E55" s="13"/>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="10"/>
-      <c r="B56" s="11"/>
-      <c r="C56" s="13"/>
+      <c r="A56" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="B56" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C56" s="13" t="s">
+        <v>67</v>
+      </c>
       <c r="D56" s="11"/>
       <c r="E56" s="13"/>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="10"/>
-      <c r="B57" s="11"/>
-      <c r="C57" s="13"/>
+      <c r="A57" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B57" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C57" s="13" t="s">
+        <v>69</v>
+      </c>
       <c r="D57" s="11"/>
       <c r="E57" s="13"/>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="10"/>
-      <c r="B58" s="11"/>
-      <c r="C58" s="13"/>
+      <c r="A58" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="B58" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C58" s="13" t="s">
+        <v>71</v>
+      </c>
       <c r="D58" s="11"/>
       <c r="E58" s="13"/>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="10"/>
-      <c r="B59" s="11"/>
-      <c r="C59" s="13"/>
+      <c r="A59" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="B59" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C59" s="13" t="s">
+        <v>73</v>
+      </c>
       <c r="D59" s="11"/>
       <c r="E59" s="13"/>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="10"/>
-      <c r="B60" s="11"/>
-      <c r="C60" s="13"/>
+      <c r="A60" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="B60" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C60" s="13" t="s">
+        <v>75</v>
+      </c>
       <c r="D60" s="11"/>
       <c r="E60" s="13"/>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="10"/>
-      <c r="B61" s="11"/>
-      <c r="C61" s="13"/>
+      <c r="A61" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="B61" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C61" s="13" t="s">
+        <v>77</v>
+      </c>
       <c r="D61" s="11"/>
       <c r="E61" s="13"/>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="10"/>
-      <c r="B62" s="11"/>
-      <c r="C62" s="13"/>
+      <c r="A62" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B62" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C62" s="13" t="s">
+        <v>79</v>
+      </c>
       <c r="D62" s="11"/>
       <c r="E62" s="13"/>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="10"/>
-      <c r="B63" s="11"/>
-      <c r="C63" s="13"/>
+      <c r="A63" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B63" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C63" s="13" t="s">
+        <v>81</v>
+      </c>
       <c r="D63" s="11"/>
       <c r="E63" s="13"/>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="10"/>
-      <c r="B64" s="11"/>
-      <c r="C64" s="13"/>
+      <c r="A64" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="B64" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C64" s="13" t="s">
+        <v>83</v>
+      </c>
       <c r="D64" s="11"/>
       <c r="E64" s="13"/>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="10"/>
-      <c r="B65" s="11"/>
-      <c r="C65" s="13"/>
+      <c r="A65" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="B65" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C65" s="13" t="s">
+        <v>85</v>
+      </c>
       <c r="D65" s="11"/>
       <c r="E65" s="13"/>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="10"/>
-      <c r="B66" s="11"/>
-      <c r="C66" s="13"/>
+      <c r="A66" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="B66" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C66" s="13" t="s">
+        <v>87</v>
+      </c>
       <c r="D66" s="11"/>
       <c r="E66" s="13"/>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="10"/>
-      <c r="B67" s="11"/>
-      <c r="C67" s="13"/>
+      <c r="A67" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="B67" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C67" s="13" t="s">
+        <v>89</v>
+      </c>
       <c r="D67" s="11"/>
       <c r="E67" s="13"/>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="18"/>
-      <c r="B68" s="11"/>
-      <c r="C68" s="13"/>
+      <c r="A68" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B68" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C68" s="13" t="s">
+        <v>91</v>
+      </c>
       <c r="D68" s="11"/>
       <c r="E68" s="13"/>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="18"/>
-      <c r="B69" s="11"/>
-      <c r="C69" s="13"/>
+      <c r="A69" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="B69" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C69" s="13" t="s">
+        <v>93</v>
+      </c>
       <c r="D69" s="11"/>
       <c r="E69" s="13"/>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="18"/>
-      <c r="B70" s="11"/>
-      <c r="C70" s="13"/>
+      <c r="A70" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="B70" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C70" s="13" t="s">
+        <v>95</v>
+      </c>
       <c r="D70" s="11"/>
       <c r="E70" s="13"/>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B71" s="11"/>
-      <c r="C71" s="11"/>
+      <c r="A71" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="B71" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C71" s="11" t="s">
+        <v>97</v>
+      </c>
       <c r="D71" s="11"/>
       <c r="E71" s="11"/>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B72" s="11"/>
-      <c r="C72" s="11"/>
+      <c r="A72" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="B72" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C72" s="11" t="s">
+        <v>99</v>
+      </c>
       <c r="D72" s="11"/>
       <c r="E72" s="11"/>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B73" s="11"/>
-      <c r="C73" s="11"/>
+      <c r="A73" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C73" s="11" t="s">
+        <v>101</v>
+      </c>
       <c r="D73" s="11"/>
       <c r="E73" s="11"/>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B74" s="11"/>
-      <c r="C74" s="11"/>
+      <c r="A74" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="B74" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C74" s="11" t="s">
+        <v>103</v>
+      </c>
       <c r="D74" s="11"/>
       <c r="E74" s="11"/>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B75" s="11"/>
-      <c r="C75" s="11"/>
+      <c r="A75" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="B75" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C75" s="11" t="s">
+        <v>105</v>
+      </c>
       <c r="D75" s="11"/>
       <c r="E75" s="11"/>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B76" s="11"/>
-      <c r="C76" s="11"/>
+      <c r="A76" s="18" t="s">
+        <v>106</v>
+      </c>
+      <c r="B76" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C76" s="11" t="s">
+        <v>107</v>
+      </c>
       <c r="D76" s="11"/>
       <c r="E76" s="11"/>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B77" s="11"/>
-      <c r="C77" s="11"/>
+      <c r="A77" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="B77" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C77" s="11" t="s">
+        <v>109</v>
+      </c>
       <c r="D77" s="11"/>
       <c r="E77" s="11"/>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B78" s="11"/>
-      <c r="C78" s="11"/>
+      <c r="A78" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="B78" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C78" s="11" t="s">
+        <v>111</v>
+      </c>
       <c r="D78" s="11"/>
       <c r="E78" s="11"/>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B79" s="11"/>
-      <c r="C79" s="11"/>
+      <c r="A79" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="B79" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C79" s="11" t="s">
+        <v>113</v>
+      </c>
       <c r="D79" s="11"/>
       <c r="E79" s="11"/>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B80" s="11"/>
-      <c r="C80" s="11"/>
+      <c r="A80" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="B80" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C80" s="11" t="s">
+        <v>115</v>
+      </c>
       <c r="D80" s="11"/>
       <c r="E80" s="11"/>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B81" s="11"/>
-      <c r="C81" s="11"/>
+      <c r="A81" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="B81" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C81" s="11" t="s">
+        <v>117</v>
+      </c>
       <c r="D81" s="11"/>
       <c r="E81" s="11"/>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B82" s="11"/>
-      <c r="C82" s="11"/>
+      <c r="A82" s="18" t="s">
+        <v>118</v>
+      </c>
+      <c r="B82" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C82" s="11" t="s">
+        <v>119</v>
+      </c>
       <c r="D82" s="11"/>
       <c r="E82" s="11"/>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B83" s="11"/>
-      <c r="C83" s="11"/>
+      <c r="A83" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="B83" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C83" s="11" t="s">
+        <v>121</v>
+      </c>
       <c r="D83" s="11"/>
       <c r="E83" s="11"/>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B84" s="11"/>
-      <c r="C84" s="11"/>
+      <c r="A84" s="18" t="s">
+        <v>122</v>
+      </c>
+      <c r="B84" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C84" s="11" t="s">
+        <v>123</v>
+      </c>
       <c r="D84" s="11"/>
       <c r="E84" s="11"/>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B85" s="11"/>
-      <c r="C85" s="11"/>
+      <c r="A85" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="B85" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C85" s="11" t="s">
+        <v>125</v>
+      </c>
       <c r="D85" s="11"/>
       <c r="E85" s="11"/>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B86" s="11"/>
-      <c r="C86" s="11"/>
+      <c r="A86" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="B86" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C86" s="11" t="s">
+        <v>127</v>
+      </c>
       <c r="D86" s="11"/>
       <c r="E86" s="11"/>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B87" s="11"/>
-      <c r="C87" s="11"/>
+      <c r="A87" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="B87" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C87" s="11" t="s">
+        <v>129</v>
+      </c>
       <c r="D87" s="11"/>
       <c r="E87" s="11"/>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B88" s="11"/>
-      <c r="C88" s="11"/>
+      <c r="A88" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="B88" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C88" s="11" t="s">
+        <v>131</v>
+      </c>
       <c r="D88" s="11"/>
       <c r="E88" s="11"/>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B89" s="11"/>
-      <c r="C89" s="11"/>
+      <c r="A89" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="B89" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C89" s="11" t="s">
+        <v>133</v>
+      </c>
       <c r="D89" s="11"/>
       <c r="E89" s="11"/>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B90" s="11"/>
-      <c r="C90" s="11"/>
+      <c r="A90" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="B90" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C90" s="11" t="s">
+        <v>135</v>
+      </c>
       <c r="D90" s="11"/>
       <c r="E90" s="11"/>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B91" s="11"/>
-      <c r="C91" s="11"/>
+      <c r="A91" s="18" t="s">
+        <v>136</v>
+      </c>
+      <c r="B91" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C91" s="11" t="s">
+        <v>137</v>
+      </c>
       <c r="D91" s="11"/>
       <c r="E91" s="11"/>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B92" s="11"/>
-      <c r="C92" s="11"/>
+      <c r="A92" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="B92" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C92" s="11" t="s">
+        <v>139</v>
+      </c>
       <c r="D92" s="11"/>
       <c r="E92" s="11"/>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B93" s="11"/>
-      <c r="C93" s="11"/>
+      <c r="A93" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="B93" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C93" s="11" t="s">
+        <v>141</v>
+      </c>
       <c r="D93" s="11"/>
       <c r="E93" s="11"/>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B94" s="11"/>
-      <c r="C94" s="11"/>
+      <c r="A94" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="B94" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C94" s="11" t="s">
+        <v>143</v>
+      </c>
       <c r="D94" s="11"/>
       <c r="E94" s="11"/>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B95" s="11"/>
-      <c r="C95" s="11"/>
+      <c r="A95" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="B95" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C95" s="11" t="s">
+        <v>145</v>
+      </c>
       <c r="D95" s="11"/>
       <c r="E95" s="11"/>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B96" s="11"/>
-      <c r="C96" s="11"/>
+      <c r="A96" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="B96" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C96" s="11" t="s">
+        <v>147</v>
+      </c>
       <c r="D96" s="11"/>
       <c r="E96" s="11"/>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B97" s="11"/>
-      <c r="C97" s="11"/>
+      <c r="A97" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="B97" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C97" s="11" t="s">
+        <v>149</v>
+      </c>
       <c r="D97" s="11"/>
       <c r="E97" s="11"/>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B98" s="11"/>
-      <c r="C98" s="11"/>
+      <c r="A98" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="B98" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C98" s="11" t="s">
+        <v>151</v>
+      </c>
       <c r="D98" s="11"/>
       <c r="E98" s="11"/>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B99" s="11"/>
-      <c r="C99" s="11"/>
+      <c r="A99" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="B99" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C99" s="11" t="s">
+        <v>153</v>
+      </c>
       <c r="D99" s="11"/>
       <c r="E99" s="11"/>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B100" s="11"/>
-      <c r="C100" s="11"/>
+      <c r="A100" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="B100" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C100" s="11" t="s">
+        <v>155</v>
+      </c>
       <c r="D100" s="11"/>
       <c r="E100" s="11"/>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B101" s="11"/>
-      <c r="C101" s="11"/>
+      <c r="A101" s="18" t="s">
+        <v>156</v>
+      </c>
+      <c r="B101" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C101" s="11" t="s">
+        <v>157</v>
+      </c>
       <c r="D101" s="11"/>
       <c r="E101" s="11"/>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B102" s="11"/>
-      <c r="C102" s="11"/>
+      <c r="A102" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="B102" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C102" s="11" t="s">
+        <v>159</v>
+      </c>
       <c r="D102" s="11"/>
       <c r="E102" s="11"/>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B103" s="11"/>
-      <c r="C103" s="11"/>
+      <c r="A103" s="18" t="s">
+        <v>160</v>
+      </c>
+      <c r="B103" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C103" s="11" t="s">
+        <v>161</v>
+      </c>
       <c r="D103" s="11"/>
       <c r="E103" s="11"/>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A104" s="18"/>
       <c r="B104" s="11"/>
       <c r="C104" s="11"/>
       <c r="D104" s="11"/>
       <c r="E104" s="11"/>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A105" s="18"/>
       <c r="B105" s="11"/>
       <c r="C105" s="11"/>
       <c r="D105" s="11"/>
       <c r="E105" s="11"/>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A106" s="18"/>
       <c r="B106" s="11"/>
       <c r="C106" s="11"/>
       <c r="D106" s="11"/>
       <c r="E106" s="11"/>
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A107" s="18"/>
       <c r="B107" s="11"/>
       <c r="C107" s="11"/>
       <c r="D107" s="11"/>
       <c r="E107" s="11"/>
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A108" s="18"/>
       <c r="B108" s="11"/>
       <c r="C108" s="11"/>
       <c r="D108" s="11"/>
       <c r="E108" s="11"/>
     </row>
     <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A109" s="18"/>
       <c r="B109" s="11"/>
       <c r="C109" s="11"/>
       <c r="D109" s="11"/>
       <c r="E109" s="11"/>
     </row>
     <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A110" s="18"/>
       <c r="B110" s="11"/>
       <c r="C110" s="11"/>
       <c r="D110" s="11"/>
       <c r="E110" s="11"/>
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A111" s="18"/>
       <c r="B111" s="11"/>
       <c r="C111" s="11"/>
       <c r="D111" s="11"/>
       <c r="E111" s="11"/>
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A112" s="18"/>
       <c r="B112" s="11"/>
       <c r="C112" s="11"/>
       <c r="D112" s="11"/>
       <c r="E112" s="11"/>
     </row>
     <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A113" s="18"/>
       <c r="B113" s="11"/>
       <c r="C113" s="11"/>
       <c r="D113" s="11"/>
       <c r="E113" s="11"/>
     </row>
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A114" s="18"/>
       <c r="B114" s="11"/>
       <c r="C114" s="11"/>
       <c r="D114" s="11"/>
       <c r="E114" s="11"/>
     </row>
     <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A115" s="18"/>
       <c r="B115" s="11"/>
       <c r="C115" s="11"/>
       <c r="D115" s="11"/>
       <c r="E115" s="11"/>
     </row>
     <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A116" s="18"/>
       <c r="B116" s="11"/>
       <c r="C116" s="11"/>
       <c r="D116" s="11"/>
       <c r="E116" s="11"/>
     </row>
     <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A117" s="18"/>
       <c r="B117" s="11"/>
       <c r="C117" s="11"/>
       <c r="D117" s="11"/>
       <c r="E117" s="11"/>
     </row>
     <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A118" s="18"/>
       <c r="B118" s="11"/>
       <c r="C118" s="11"/>
       <c r="D118" s="11"/>
       <c r="E118" s="11"/>
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A119" s="18"/>
       <c r="B119" s="11"/>
       <c r="C119" s="11"/>
       <c r="D119" s="11"/>
       <c r="E119" s="11"/>
     </row>
     <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A120" s="18"/>
       <c r="B120" s="11"/>
       <c r="C120" s="11"/>
       <c r="D120" s="11"/>
       <c r="E120" s="11"/>
     </row>
     <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A121" s="18"/>
       <c r="B121" s="11"/>
       <c r="C121" s="11"/>
       <c r="D121" s="11"/>
       <c r="E121" s="11"/>
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A122" s="18"/>
       <c r="B122" s="11"/>
       <c r="C122" s="11"/>
       <c r="D122" s="11"/>
       <c r="E122" s="11"/>
     </row>
     <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A123" s="18"/>
       <c r="B123" s="11"/>
       <c r="C123" s="11"/>
       <c r="D123" s="11"/>
       <c r="E123" s="11"/>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A124" s="18"/>
       <c r="B124" s="11"/>
       <c r="C124" s="11"/>
       <c r="D124" s="11"/>
       <c r="E124" s="11"/>
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A125" s="18"/>
       <c r="B125" s="11"/>
       <c r="C125" s="11"/>
       <c r="D125" s="11"/>
       <c r="E125" s="11"/>
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A126" s="18"/>
       <c r="B126" s="11"/>
       <c r="C126" s="11"/>
       <c r="D126" s="11"/>
       <c r="E126" s="11"/>
     </row>
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A127" s="18"/>
       <c r="B127" s="11"/>
       <c r="C127" s="11"/>
       <c r="D127" s="11"/>
       <c r="E127" s="11"/>
     </row>
     <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A128" s="18"/>
       <c r="B128" s="11"/>
       <c r="C128" s="11"/>
       <c r="D128" s="11"/>
       <c r="E128" s="11"/>
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A129" s="18"/>
       <c r="B129" s="11"/>
       <c r="C129" s="11"/>
       <c r="D129" s="11"/>
       <c r="E129" s="11"/>
     </row>
     <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A130" s="18"/>
       <c r="B130" s="11"/>
       <c r="C130" s="11"/>
       <c r="D130" s="11"/>
       <c r="E130" s="11"/>
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A131" s="18"/>
       <c r="B131" s="11"/>
       <c r="C131" s="11"/>
       <c r="D131" s="11"/>
       <c r="E131" s="11"/>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A132" s="18"/>
       <c r="B132" s="11"/>
       <c r="C132" s="11"/>
       <c r="D132" s="11"/>
       <c r="E132" s="11"/>
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A133" s="18"/>
       <c r="B133" s="11"/>
       <c r="C133" s="11"/>
       <c r="D133" s="11"/>
       <c r="E133" s="11"/>
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A134" s="18"/>
       <c r="B134" s="11"/>
       <c r="C134" s="11"/>
       <c r="D134" s="11"/>
       <c r="E134" s="11"/>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A135" s="18"/>
       <c r="B135" s="11"/>
       <c r="C135" s="11"/>
       <c r="D135" s="11"/>
       <c r="E135" s="11"/>
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A136" s="18"/>
       <c r="B136" s="11"/>
       <c r="C136" s="11"/>
       <c r="D136" s="11"/>
       <c r="E136" s="11"/>
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A137" s="18"/>
       <c r="B137" s="11"/>
       <c r="C137" s="11"/>
       <c r="D137" s="11"/>
       <c r="E137" s="11"/>
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A138" s="18"/>
       <c r="B138" s="11"/>
       <c r="C138" s="11"/>
       <c r="D138" s="11"/>
       <c r="E138" s="11"/>
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A139" s="18"/>
       <c r="B139" s="11"/>
       <c r="C139" s="11"/>
       <c r="D139" s="11"/>
       <c r="E139" s="11"/>
     </row>
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A140" s="18"/>
       <c r="B140" s="11"/>
       <c r="C140" s="11"/>
       <c r="D140" s="11"/>
       <c r="E140" s="11"/>
     </row>
     <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A141" s="18"/>
       <c r="B141" s="11"/>
       <c r="C141" s="11"/>
       <c r="D141" s="11"/>
       <c r="E141" s="11"/>
     </row>
     <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A142" s="18"/>
       <c r="B142" s="11"/>
       <c r="C142" s="11"/>
       <c r="D142" s="11"/>
       <c r="E142" s="11"/>
     </row>
     <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A143" s="18"/>
       <c r="B143" s="11"/>
       <c r="C143" s="11"/>
       <c r="D143" s="11"/>
       <c r="E143" s="11"/>
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A144" s="18"/>
       <c r="B144" s="11"/>
       <c r="C144" s="11"/>
       <c r="D144" s="11"/>
       <c r="E144" s="11"/>
     </row>
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A145" s="18"/>
       <c r="B145" s="11"/>
       <c r="C145" s="11"/>
       <c r="D145" s="11"/>
       <c r="E145" s="11"/>
     </row>
     <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A146" s="18"/>
       <c r="B146" s="11"/>
       <c r="C146" s="11"/>
       <c r="D146" s="11"/>
       <c r="E146" s="11"/>
     </row>
     <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A147" s="18"/>
       <c r="B147" s="11"/>
       <c r="C147" s="11"/>
       <c r="D147" s="11"/>
       <c r="E147" s="11"/>
     </row>
     <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A148" s="18"/>
       <c r="B148" s="11"/>
       <c r="C148" s="11"/>
       <c r="D148" s="11"/>
       <c r="E148" s="11"/>
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A149" s="18"/>
       <c r="B149" s="11"/>
       <c r="C149" s="11"/>
       <c r="D149" s="11"/>
       <c r="E149" s="11"/>
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A150" s="18"/>
       <c r="B150" s="11"/>
       <c r="C150" s="11"/>
       <c r="D150" s="11"/>
       <c r="E150" s="11"/>
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A151" s="18"/>
       <c r="B151" s="11"/>
       <c r="C151" s="11"/>
       <c r="D151" s="11"/>
       <c r="E151" s="11"/>
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A152" s="18"/>
       <c r="B152" s="11"/>
       <c r="C152" s="11"/>
       <c r="D152" s="11"/>
       <c r="E152" s="11"/>
     </row>
     <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A153" s="18"/>
       <c r="B153" s="11"/>
       <c r="C153" s="11"/>
       <c r="D153" s="11"/>
       <c r="E153" s="11"/>
     </row>
     <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A154" s="18"/>
       <c r="B154" s="11"/>
       <c r="C154" s="11"/>
       <c r="D154" s="11"/>
       <c r="E154" s="11"/>
     </row>
     <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A155" s="18"/>
       <c r="B155" s="11"/>
       <c r="C155" s="11"/>
       <c r="D155" s="11"/>
       <c r="E155" s="11"/>
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A156" s="18"/>
       <c r="B156" s="11"/>
       <c r="C156" s="11"/>
       <c r="D156" s="11"/>
       <c r="E156" s="11"/>
     </row>
     <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A157" s="18"/>
       <c r="B157" s="11"/>
       <c r="C157" s="11"/>
       <c r="D157" s="11"/>
       <c r="E157" s="11"/>
     </row>
     <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A158" s="18"/>
       <c r="B158" s="11"/>
       <c r="C158" s="11"/>
       <c r="D158" s="11"/>
       <c r="E158" s="11"/>
     </row>
     <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A159" s="18"/>
       <c r="B159" s="11"/>
       <c r="C159" s="11"/>
       <c r="D159" s="11"/>
       <c r="E159" s="11"/>
     </row>
     <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A160" s="18"/>
       <c r="B160" s="11"/>
       <c r="C160" s="11"/>
       <c r="D160" s="11"/>
       <c r="E160" s="11"/>
     </row>
     <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A161" s="18"/>
       <c r="B161" s="11"/>
       <c r="C161" s="11"/>
       <c r="D161" s="11"/>
       <c r="E161" s="11"/>
     </row>
     <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A162" s="18"/>
       <c r="B162" s="11"/>
       <c r="C162" s="11"/>
       <c r="D162" s="11"/>
       <c r="E162" s="11"/>
     </row>
     <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A163" s="18"/>
       <c r="B163" s="11"/>
       <c r="C163" s="11"/>
       <c r="D163" s="11"/>
       <c r="E163" s="11"/>
     </row>
     <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A164" s="18"/>
       <c r="B164" s="11"/>
       <c r="C164" s="11"/>
       <c r="D164" s="11"/>
       <c r="E164" s="11"/>
     </row>
     <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A165" s="18"/>
       <c r="B165" s="11"/>
       <c r="C165" s="11"/>
       <c r="D165" s="11"/>
       <c r="E165" s="11"/>
     </row>
     <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A166" s="18"/>
       <c r="B166" s="11"/>
       <c r="C166" s="11"/>
       <c r="D166" s="11"/>
       <c r="E166" s="11"/>
     </row>
     <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A167" s="18"/>
       <c r="B167" s="11"/>
       <c r="C167" s="11"/>
       <c r="D167" s="11"/>
       <c r="E167" s="11"/>
     </row>
     <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A168" s="18"/>
       <c r="B168" s="11"/>
       <c r="C168" s="11"/>
       <c r="D168" s="11"/>
       <c r="E168" s="11"/>
     </row>
     <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A169" s="18"/>
       <c r="B169" s="11"/>
       <c r="C169" s="11"/>
       <c r="D169" s="11"/>
       <c r="E169" s="11"/>
     </row>
     <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A170" s="18"/>
       <c r="B170" s="11"/>
       <c r="C170" s="11"/>
       <c r="D170" s="11"/>
       <c r="E170" s="11"/>
     </row>
     <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A171" s="18"/>
       <c r="B171" s="11"/>
       <c r="C171" s="11"/>
       <c r="D171" s="11"/>
       <c r="E171" s="11"/>
     </row>
     <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A172" s="18"/>
       <c r="B172" s="11"/>
       <c r="C172" s="11"/>
       <c r="D172" s="11"/>
       <c r="E172" s="11"/>
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A173" s="18"/>
       <c r="B173" s="11"/>
       <c r="C173" s="11"/>
       <c r="D173" s="11"/>
       <c r="E173" s="11"/>
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A174" s="18"/>
       <c r="B174" s="11"/>
       <c r="C174" s="11"/>
       <c r="D174" s="11"/>
       <c r="E174" s="11"/>
     </row>
     <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A175" s="18"/>
       <c r="B175" s="11"/>
       <c r="C175" s="11"/>
       <c r="D175" s="11"/>
       <c r="E175" s="11"/>
     </row>
     <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A176" s="18"/>
       <c r="B176" s="11"/>
       <c r="C176" s="11"/>
       <c r="D176" s="11"/>
       <c r="E176" s="11"/>
     </row>
     <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A177" s="18"/>
       <c r="B177" s="11"/>
       <c r="C177" s="11"/>
       <c r="D177" s="11"/>
       <c r="E177" s="11"/>
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A178" s="18"/>
       <c r="B178" s="11"/>
       <c r="C178" s="11"/>
       <c r="D178" s="11"/>
       <c r="E178" s="11"/>
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A179" s="18"/>
       <c r="B179" s="11"/>
       <c r="C179" s="11"/>
       <c r="D179" s="11"/>
       <c r="E179" s="11"/>
     </row>
     <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A180" s="18"/>
       <c r="B180" s="11"/>
       <c r="C180" s="11"/>
       <c r="D180" s="11"/>
       <c r="E180" s="11"/>
     </row>
     <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A181" s="18"/>
       <c r="B181" s="11"/>
       <c r="C181" s="11"/>
       <c r="D181" s="11"/>
       <c r="E181" s="11"/>
     </row>
     <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A182" s="18"/>
       <c r="B182" s="11"/>
       <c r="C182" s="11"/>
       <c r="D182" s="11"/>
       <c r="E182" s="11"/>
     </row>
     <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A183" s="18"/>
       <c r="B183" s="11"/>
       <c r="C183" s="11"/>
       <c r="D183" s="11"/>
       <c r="E183" s="11"/>
     </row>
     <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A184" s="18"/>
       <c r="B184" s="11"/>
       <c r="C184" s="11"/>
       <c r="D184" s="11"/>
       <c r="E184" s="11"/>
     </row>
     <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A185" s="18"/>
       <c r="B185" s="11"/>
       <c r="C185" s="11"/>
       <c r="D185" s="11"/>
       <c r="E185" s="11"/>
     </row>
     <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A186" s="18"/>
       <c r="B186" s="11"/>
       <c r="C186" s="11"/>
       <c r="D186" s="11"/>
       <c r="E186" s="11"/>
     </row>
     <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A187" s="18"/>
       <c r="B187" s="11"/>
       <c r="C187" s="11"/>
       <c r="D187" s="11"/>
       <c r="E187" s="11"/>
     </row>
     <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A188" s="18"/>
       <c r="B188" s="11"/>
       <c r="C188" s="11"/>
       <c r="D188" s="11"/>
       <c r="E188" s="11"/>
     </row>
     <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A189" s="18"/>
       <c r="B189" s="11"/>
       <c r="C189" s="11"/>
       <c r="D189" s="11"/>
       <c r="E189" s="11"/>
     </row>
     <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A190" s="18"/>
       <c r="B190" s="11"/>
       <c r="C190" s="11"/>
       <c r="D190" s="11"/>
       <c r="E190" s="11"/>
     </row>
     <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A191" s="18"/>
       <c r="B191" s="11"/>
       <c r="C191" s="11"/>
       <c r="D191" s="11"/>
       <c r="E191" s="11"/>
     </row>
     <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A192" s="18"/>
       <c r="B192" s="11"/>
       <c r="C192" s="11"/>
       <c r="D192" s="11"/>
       <c r="E192" s="11"/>
     </row>
     <row r="193" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A193" s="18"/>
       <c r="B193" s="11"/>
       <c r="C193" s="11"/>
       <c r="D193" s="11"/>
       <c r="E193" s="11"/>
     </row>
     <row r="194" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A194" s="18"/>
       <c r="B194" s="11"/>
       <c r="C194" s="11"/>
       <c r="D194" s="11"/>
       <c r="E194" s="11"/>
     </row>
     <row r="195" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A195" s="18"/>
       <c r="B195" s="11"/>
       <c r="C195" s="11"/>
       <c r="D195" s="11"/>
       <c r="E195" s="11"/>
     </row>
     <row r="196" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A196" s="18"/>
       <c r="B196" s="11"/>
       <c r="C196" s="11"/>
       <c r="D196" s="11"/>
       <c r="E196" s="11"/>
     </row>
     <row r="197" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A197" s="18"/>
       <c r="B197" s="11"/>
       <c r="C197" s="11"/>
       <c r="D197" s="11"/>
       <c r="E197" s="11"/>
     </row>
     <row r="198" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A198" s="18"/>
       <c r="B198" s="11"/>
       <c r="C198" s="11"/>
       <c r="D198" s="11"/>
       <c r="E198" s="11"/>
     </row>
     <row r="199" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A199" s="18"/>
       <c r="B199" s="11"/>
       <c r="C199" s="11"/>
       <c r="D199" s="11"/>
       <c r="E199" s="11"/>
     </row>
     <row r="200" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A200" s="18"/>
       <c r="B200" s="11"/>
       <c r="C200" s="11"/>
       <c r="D200" s="11"/>
       <c r="E200" s="11"/>
     </row>
     <row r="201" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A201" s="18"/>
       <c r="B201" s="11"/>
       <c r="C201" s="11"/>
       <c r="D201" s="11"/>
       <c r="E201" s="11"/>
     </row>
     <row r="202" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A202" s="18"/>
       <c r="B202" s="11"/>
       <c r="C202" s="11"/>
       <c r="D202" s="11"/>
       <c r="E202" s="11"/>
     </row>
     <row r="203" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A203" s="18"/>
       <c r="B203" s="11"/>
       <c r="C203" s="11"/>
       <c r="D203" s="11"/>
       <c r="E203" s="11"/>
     </row>
     <row r="204" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A204" s="18"/>
       <c r="B204" s="11"/>
       <c r="C204" s="11"/>
       <c r="D204" s="11"/>
       <c r="E204" s="11"/>
     </row>
     <row r="205" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A205" s="18"/>
       <c r="B205" s="11"/>
       <c r="C205" s="11"/>
       <c r="D205" s="11"/>
       <c r="E205" s="11"/>
     </row>
     <row r="206" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A206" s="18"/>
       <c r="B206" s="11"/>
       <c r="C206" s="11"/>
       <c r="D206" s="11"/>
       <c r="E206" s="11"/>
     </row>
     <row r="207" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A207" s="18"/>
       <c r="B207" s="11"/>
       <c r="C207" s="11"/>
       <c r="D207" s="11"/>
       <c r="E207" s="11"/>
     </row>
     <row r="208" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A208" s="18"/>
       <c r="B208" s="11"/>
       <c r="C208" s="11"/>
       <c r="D208" s="11"/>
       <c r="E208" s="11"/>
     </row>
     <row r="209" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A209" s="18"/>
       <c r="B209" s="11"/>
       <c r="C209" s="11"/>
       <c r="D209" s="11"/>
       <c r="E209" s="11"/>
     </row>
     <row r="210" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A210" s="18"/>
       <c r="B210" s="11"/>
       <c r="C210" s="11"/>
       <c r="D210" s="11"/>
       <c r="E210" s="11"/>
     </row>
     <row r="211" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A211" s="18"/>
       <c r="B211" s="11"/>
       <c r="C211" s="11"/>
       <c r="D211" s="11"/>
       <c r="E211" s="11"/>
     </row>
     <row r="212" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A212" s="18"/>
       <c r="B212" s="11"/>
       <c r="C212" s="11"/>
       <c r="D212" s="11"/>
       <c r="E212" s="11"/>
     </row>
     <row r="213" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A213" s="18"/>
       <c r="B213" s="11"/>
       <c r="C213" s="11"/>
       <c r="D213" s="11"/>
       <c r="E213" s="11"/>
     </row>
     <row r="214" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A214" s="18"/>
       <c r="B214" s="11"/>
       <c r="C214" s="11"/>
       <c r="D214" s="11"/>
       <c r="E214" s="11"/>
     </row>
     <row r="215" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A215" s="18"/>
       <c r="B215" s="11"/>
       <c r="C215" s="11"/>
       <c r="D215" s="11"/>
       <c r="E215" s="11"/>
     </row>
     <row r="216" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A216" s="18"/>
       <c r="B216" s="11"/>
       <c r="C216" s="11"/>
       <c r="D216" s="11"/>
       <c r="E216" s="11"/>
     </row>
     <row r="217" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A217" s="18"/>
       <c r="B217" s="11"/>
       <c r="C217" s="11"/>
       <c r="D217" s="11"/>
       <c r="E217" s="11"/>
     </row>
     <row r="218" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A218" s="18"/>
       <c r="B218" s="11"/>
       <c r="C218" s="11"/>
       <c r="D218" s="11"/>
       <c r="E218" s="11"/>
     </row>
     <row r="219" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A219" s="18"/>
       <c r="B219" s="11"/>
       <c r="C219" s="11"/>
       <c r="D219" s="11"/>
       <c r="E219" s="11"/>
     </row>
     <row r="220" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A220" s="18"/>
       <c r="B220" s="11"/>
       <c r="C220" s="11"/>
       <c r="D220" s="11"/>
       <c r="E220" s="11"/>
     </row>
     <row r="221" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A221" s="18"/>
       <c r="B221" s="11"/>
       <c r="C221" s="11"/>
       <c r="D221" s="11"/>
       <c r="E221" s="11"/>
     </row>
     <row r="222" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A222" s="18"/>
       <c r="B222" s="11"/>
       <c r="C222" s="11"/>
       <c r="D222" s="11"/>
       <c r="E222" s="11"/>
     </row>
     <row r="223" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A223" s="18"/>
       <c r="B223" s="11"/>
       <c r="C223" s="11"/>
       <c r="D223" s="11"/>
       <c r="E223" s="11"/>
     </row>
     <row r="224" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A224" s="18"/>
       <c r="B224" s="11"/>
       <c r="C224" s="11"/>
       <c r="D224" s="11"/>
       <c r="E224" s="11"/>
     </row>
     <row r="225" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A225" s="18"/>
       <c r="B225" s="11"/>
       <c r="C225" s="11"/>
       <c r="D225" s="11"/>
       <c r="E225" s="11"/>
     </row>
     <row r="226" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A226" s="18"/>
       <c r="B226" s="11"/>
       <c r="C226" s="11"/>
       <c r="D226" s="11"/>
       <c r="E226" s="11"/>
     </row>
     <row r="227" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A227" s="18"/>
       <c r="B227" s="11"/>
       <c r="C227" s="11"/>
       <c r="D227" s="11"/>
       <c r="E227" s="11"/>
     </row>
     <row r="228" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A228" s="18"/>
       <c r="B228" s="11"/>
       <c r="C228" s="11"/>
       <c r="D228" s="11"/>
       <c r="E228" s="11"/>
     </row>
     <row r="229" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A229" s="18"/>
       <c r="B229" s="11"/>
       <c r="C229" s="11"/>
       <c r="D229" s="11"/>
       <c r="E229" s="11"/>
     </row>
     <row r="230" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A230" s="18"/>
       <c r="B230" s="11"/>
       <c r="C230" s="11"/>
       <c r="D230" s="11"/>
       <c r="E230" s="11"/>
     </row>
     <row r="231" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A231" s="18"/>
       <c r="B231" s="11"/>
       <c r="C231" s="11"/>
       <c r="D231" s="11"/>
       <c r="E231" s="11"/>
     </row>
     <row r="232" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A232" s="18"/>
       <c r="B232" s="11"/>
       <c r="C232" s="11"/>
       <c r="D232" s="11"/>
       <c r="E232" s="11"/>
     </row>
     <row r="233" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A233" s="18"/>
       <c r="B233" s="11"/>
       <c r="C233" s="11"/>
       <c r="D233" s="11"/>
       <c r="E233" s="11"/>
     </row>
     <row r="234" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A234" s="18"/>
       <c r="B234" s="11"/>
       <c r="C234" s="11"/>
       <c r="D234" s="11"/>
       <c r="E234" s="11"/>
     </row>
     <row r="235" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A235" s="18"/>
       <c r="B235" s="11"/>
       <c r="C235" s="11"/>
       <c r="D235" s="11"/>
       <c r="E235" s="11"/>
     </row>
     <row r="236" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A236" s="18"/>
       <c r="B236" s="11"/>
       <c r="C236" s="11"/>
       <c r="D236" s="11"/>
       <c r="E236" s="11"/>
     </row>
     <row r="237" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A237" s="18"/>
       <c r="B237" s="11"/>
       <c r="C237" s="11"/>
       <c r="D237" s="11"/>
       <c r="E237" s="11"/>
     </row>
     <row r="238" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A238" s="18"/>
       <c r="B238" s="11"/>
       <c r="C238" s="11"/>
       <c r="D238" s="11"/>
       <c r="E238" s="11"/>
     </row>
     <row r="239" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A239" s="18"/>
       <c r="B239" s="11"/>
       <c r="C239" s="11"/>
       <c r="D239" s="11"/>
       <c r="E239" s="11"/>
     </row>
     <row r="240" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A240" s="18"/>
       <c r="B240" s="11"/>
       <c r="C240" s="11"/>
       <c r="D240" s="11"/>
       <c r="E240" s="11"/>
     </row>
     <row r="241" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A241" s="18"/>
       <c r="B241" s="11"/>
       <c r="C241" s="11"/>
       <c r="D241" s="11"/>
       <c r="E241" s="11"/>
     </row>
     <row r="242" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A242" s="18"/>
       <c r="B242" s="11"/>
       <c r="C242" s="11"/>
       <c r="D242" s="11"/>
       <c r="E242" s="11"/>
     </row>
     <row r="243" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A243" s="18"/>
       <c r="B243" s="11"/>
       <c r="C243" s="11"/>
       <c r="D243" s="11"/>
       <c r="E243" s="11"/>
     </row>
     <row r="244" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A244" s="18"/>
       <c r="B244" s="11"/>
       <c r="C244" s="11"/>
       <c r="D244" s="11"/>
       <c r="E244" s="11"/>
     </row>
     <row r="245" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A245" s="18"/>
       <c r="B245" s="11"/>
       <c r="C245" s="11"/>
       <c r="D245" s="11"/>
       <c r="E245" s="11"/>
     </row>
     <row r="246" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A246" s="18"/>
       <c r="B246" s="11"/>
       <c r="C246" s="11"/>
       <c r="D246" s="11"/>
       <c r="E246" s="11"/>
     </row>
     <row r="247" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A247" s="18"/>
       <c r="B247" s="11"/>
       <c r="C247" s="11"/>
       <c r="D247" s="11"/>
       <c r="E247" s="11"/>
     </row>
     <row r="248" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A248" s="18"/>
       <c r="B248" s="11"/>
       <c r="C248" s="11"/>
       <c r="D248" s="11"/>
       <c r="E248" s="11"/>
     </row>
     <row r="249" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A249" s="18"/>
       <c r="B249" s="11"/>
       <c r="C249" s="11"/>
       <c r="D249" s="11"/>
       <c r="E249" s="11"/>
     </row>
     <row r="250" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A250" s="18"/>
       <c r="B250" s="11"/>
       <c r="C250" s="11"/>
       <c r="D250" s="11"/>
       <c r="E250" s="11"/>
     </row>
     <row r="251" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A251" s="18"/>
       <c r="B251" s="11"/>
       <c r="C251" s="11"/>
       <c r="D251" s="11"/>
       <c r="E251" s="11"/>
     </row>
     <row r="252" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A252" s="18"/>
       <c r="B252" s="11"/>
       <c r="C252" s="11"/>
       <c r="D252" s="11"/>
       <c r="E252" s="11"/>
     </row>
     <row r="253" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A253" s="18"/>
       <c r="B253" s="11"/>
       <c r="C253" s="11"/>
       <c r="D253" s="11"/>
       <c r="E253" s="11"/>
     </row>
     <row r="254" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A254" s="18"/>
       <c r="B254" s="11"/>
       <c r="C254" s="11"/>
       <c r="D254" s="11"/>
       <c r="E254" s="11"/>
     </row>
     <row r="255" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A255" s="18"/>
       <c r="B255" s="11"/>
       <c r="C255" s="11"/>
       <c r="D255" s="11"/>
       <c r="E255" s="11"/>
     </row>
     <row r="256" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A256" s="18"/>
       <c r="B256" s="11"/>
       <c r="C256" s="11"/>
       <c r="D256" s="11"/>
       <c r="E256" s="11"/>
     </row>
     <row r="257" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A257" s="18"/>
       <c r="B257" s="11"/>
       <c r="C257" s="11"/>
       <c r="D257" s="11"/>
       <c r="E257" s="11"/>
     </row>
     <row r="258" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A258" s="18"/>
       <c r="B258" s="11"/>
       <c r="C258" s="11"/>
       <c r="D258" s="11"/>
       <c r="E258" s="11"/>
     </row>
     <row r="259" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A259" s="18"/>
       <c r="B259" s="11"/>
       <c r="C259" s="11"/>
       <c r="D259" s="11"/>
       <c r="E259" s="11"/>
     </row>
     <row r="260" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A260" s="18"/>
       <c r="B260" s="11"/>
       <c r="C260" s="11"/>
       <c r="D260" s="11"/>
       <c r="E260" s="11"/>
     </row>
     <row r="261" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A261" s="18"/>
       <c r="B261" s="11"/>
       <c r="C261" s="11"/>
       <c r="D261" s="11"/>
       <c r="E261" s="11"/>
     </row>
     <row r="262" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A262" s="18"/>
       <c r="B262" s="11"/>
       <c r="C262" s="11"/>
       <c r="D262" s="11"/>
       <c r="E262" s="11"/>
     </row>
     <row r="263" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A263" s="18"/>
       <c r="B263" s="11"/>
       <c r="C263" s="11"/>
       <c r="D263" s="11"/>
       <c r="E263" s="11"/>
     </row>
     <row r="264" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A264" s="18"/>
       <c r="B264" s="11"/>
       <c r="C264" s="11"/>
       <c r="D264" s="11"/>
       <c r="E264" s="11"/>
     </row>
     <row r="265" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A265" s="18"/>
       <c r="B265" s="11"/>
       <c r="C265" s="11"/>
       <c r="D265" s="11"/>
       <c r="E265" s="11"/>
     </row>
     <row r="266" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A266" s="18"/>
       <c r="B266" s="11"/>
       <c r="C266" s="11"/>
       <c r="D266" s="11"/>
       <c r="E266" s="11"/>
     </row>
     <row r="267" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A267" s="18"/>
       <c r="B267" s="11"/>
       <c r="C267" s="11"/>
       <c r="D267" s="11"/>
       <c r="E267" s="11"/>
     </row>
     <row r="268" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A268" s="18"/>
       <c r="B268" s="11"/>
       <c r="C268" s="11"/>
       <c r="D268" s="11"/>
       <c r="E268" s="11"/>
     </row>
     <row r="269" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A269" s="18"/>
       <c r="B269" s="11"/>
       <c r="C269" s="11"/>
       <c r="D269" s="11"/>
       <c r="E269" s="11"/>
     </row>
     <row r="270" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A270" s="18"/>
       <c r="B270" s="11"/>
       <c r="C270" s="11"/>
       <c r="D270" s="11"/>
       <c r="E270" s="11"/>
     </row>
     <row r="271" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A271" s="18"/>
       <c r="B271" s="11"/>
       <c r="C271" s="11"/>
       <c r="D271" s="11"/>
       <c r="E271" s="11"/>
     </row>
     <row r="272" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A272" s="18"/>
       <c r="B272" s="11"/>
       <c r="C272" s="11"/>
       <c r="D272" s="11"/>
       <c r="E272" s="11"/>
     </row>
     <row r="273" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A273" s="18"/>
       <c r="B273" s="11"/>
       <c r="C273" s="11"/>
       <c r="D273" s="11"/>
       <c r="E273" s="11"/>
     </row>
     <row r="274" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A274" s="18"/>
       <c r="B274" s="11"/>
       <c r="C274" s="11"/>
       <c r="D274" s="11"/>
       <c r="E274" s="11"/>
     </row>
     <row r="275" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A275" s="18"/>
       <c r="B275" s="11"/>
       <c r="C275" s="11"/>
       <c r="D275" s="11"/>
       <c r="E275" s="11"/>
     </row>
     <row r="276" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A276" s="18"/>
       <c r="B276" s="11"/>
       <c r="C276" s="11"/>
       <c r="D276" s="11"/>
       <c r="E276" s="11"/>
     </row>
     <row r="277" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A277" s="18"/>
       <c r="B277" s="11"/>
       <c r="C277" s="11"/>
       <c r="D277" s="11"/>
       <c r="E277" s="11"/>
     </row>
     <row r="278" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A278" s="18"/>
       <c r="B278" s="11"/>
       <c r="C278" s="11"/>
       <c r="D278" s="11"/>
       <c r="E278" s="11"/>
     </row>
     <row r="279" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A279" s="18"/>
       <c r="B279" s="11"/>
       <c r="C279" s="11"/>
       <c r="D279" s="11"/>
       <c r="E279" s="11"/>
     </row>
     <row r="280" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A280" s="18"/>
       <c r="B280" s="11"/>
       <c r="C280" s="11"/>
       <c r="D280" s="11"/>
       <c r="E280" s="11"/>
     </row>
     <row r="281" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A281" s="18"/>
       <c r="B281" s="11"/>
       <c r="C281" s="11"/>
       <c r="D281" s="11"/>
       <c r="E281" s="11"/>
     </row>
     <row r="282" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A282" s="18"/>
       <c r="B282" s="11"/>
       <c r="C282" s="11"/>
       <c r="D282" s="11"/>
       <c r="E282" s="11"/>
     </row>
     <row r="283" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A283" s="18"/>
       <c r="B283" s="11"/>
       <c r="C283" s="11"/>
       <c r="D283" s="11"/>
       <c r="E283" s="11"/>
     </row>
     <row r="284" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A284" s="18"/>
       <c r="B284" s="11"/>
       <c r="C284" s="11"/>
       <c r="D284" s="11"/>
       <c r="E284" s="11"/>
     </row>
     <row r="285" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A285" s="18"/>
       <c r="B285" s="11"/>
       <c r="C285" s="11"/>
       <c r="D285" s="11"/>
       <c r="E285" s="11"/>
     </row>
     <row r="286" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A286" s="18"/>
       <c r="B286" s="11"/>
       <c r="C286" s="11"/>
       <c r="D286" s="11"/>
       <c r="E286" s="11"/>
     </row>
     <row r="287" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A287" s="18"/>
       <c r="B287" s="11"/>
       <c r="C287" s="11"/>
       <c r="D287" s="11"/>
       <c r="E287" s="11"/>
     </row>
     <row r="288" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A288" s="18"/>
       <c r="B288" s="11"/>
       <c r="C288" s="11"/>
       <c r="D288" s="11"/>
       <c r="E288" s="11"/>
     </row>
     <row r="289" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A289" s="18"/>
       <c r="B289" s="11"/>
       <c r="C289" s="11"/>
       <c r="D289" s="11"/>
       <c r="E289" s="11"/>
     </row>
     <row r="290" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A290" s="18"/>
       <c r="B290" s="11"/>
       <c r="C290" s="11"/>
       <c r="D290" s="11"/>
       <c r="E290" s="11"/>
     </row>
     <row r="291" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A291" s="18"/>
       <c r="B291" s="11"/>
       <c r="C291" s="11"/>
       <c r="D291" s="11"/>
       <c r="E291" s="11"/>
     </row>
     <row r="292" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A292" s="18"/>
       <c r="B292" s="11"/>
       <c r="C292" s="11"/>
       <c r="D292" s="11"/>
       <c r="E292" s="11"/>
     </row>
     <row r="293" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A293" s="18"/>
       <c r="B293" s="11"/>
       <c r="C293" s="11"/>
       <c r="D293" s="11"/>
       <c r="E293" s="11"/>
     </row>
     <row r="294" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A294" s="18"/>
       <c r="B294" s="11"/>
       <c r="C294" s="11"/>
       <c r="D294" s="11"/>
       <c r="E294" s="11"/>
     </row>
     <row r="295" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A295" s="18"/>
       <c r="B295" s="11"/>
       <c r="C295" s="11"/>
       <c r="D295" s="11"/>
       <c r="E295" s="11"/>
     </row>
     <row r="296" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A296" s="18"/>
       <c r="B296" s="11"/>
       <c r="C296" s="11"/>
       <c r="D296" s="11"/>
       <c r="E296" s="11"/>
     </row>
     <row r="297" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A297" s="18"/>
       <c r="B297" s="11"/>
       <c r="C297" s="11"/>
       <c r="D297" s="11"/>
       <c r="E297" s="11"/>
     </row>
     <row r="298" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A298" s="18"/>
       <c r="B298" s="11"/>
       <c r="C298" s="11"/>
       <c r="D298" s="11"/>
       <c r="E298" s="11"/>
     </row>
     <row r="299" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A299" s="18"/>
       <c r="B299" s="11"/>
       <c r="C299" s="11"/>
       <c r="D299" s="11"/>
       <c r="E299" s="11"/>
     </row>
     <row r="300" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A300" s="18"/>
       <c r="B300" s="11"/>
       <c r="C300" s="11"/>
       <c r="D300" s="11"/>
       <c r="E300" s="11"/>
     </row>
     <row r="301" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A301" s="18"/>
       <c r="B301" s="11"/>
       <c r="C301" s="11"/>
       <c r="D301" s="11"/>
       <c r="E301" s="11"/>
     </row>
     <row r="302" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A302" s="18"/>
       <c r="B302" s="11"/>
       <c r="C302" s="11"/>
       <c r="D302" s="11"/>
       <c r="E302" s="11"/>
     </row>
     <row r="303" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A303" s="18"/>
       <c r="B303" s="11"/>
       <c r="C303" s="11"/>
       <c r="D303" s="11"/>
       <c r="E303" s="11"/>
     </row>
     <row r="304" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A304" s="18"/>
       <c r="B304" s="11"/>
       <c r="C304" s="11"/>
       <c r="D304" s="11"/>
       <c r="E304" s="11"/>
     </row>
     <row r="305" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A305" s="18"/>
       <c r="B305" s="11"/>
       <c r="C305" s="11"/>
       <c r="D305" s="11"/>
       <c r="E305" s="11"/>
     </row>
     <row r="306" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A306" s="18"/>
       <c r="B306" s="11"/>
       <c r="C306" s="11"/>
       <c r="D306" s="11"/>
       <c r="E306" s="11"/>
     </row>
     <row r="307" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A307" s="18"/>
       <c r="B307" s="11"/>
       <c r="C307" s="11"/>
       <c r="D307" s="11"/>
       <c r="E307" s="11"/>
     </row>
     <row r="308" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A308" s="18"/>
       <c r="B308" s="11"/>
       <c r="C308" s="11"/>
       <c r="D308" s="11"/>
       <c r="E308" s="11"/>
     </row>
     <row r="309" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A309" s="18"/>
       <c r="B309" s="11"/>
       <c r="C309" s="11"/>
       <c r="D309" s="11"/>
       <c r="E309" s="11"/>
     </row>
     <row r="310" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A310" s="18"/>
       <c r="B310" s="11"/>
       <c r="C310" s="11"/>
       <c r="D310" s="11"/>
       <c r="E310" s="11"/>
     </row>
     <row r="311" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A311" s="18"/>
       <c r="B311" s="11"/>
       <c r="C311" s="11"/>
       <c r="D311" s="11"/>
       <c r="E311" s="11"/>
     </row>
     <row r="312" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A312" s="18"/>
       <c r="B312" s="11"/>
       <c r="C312" s="11"/>
       <c r="D312" s="11"/>
       <c r="E312" s="11"/>
     </row>
     <row r="313" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A313" s="18"/>
       <c r="B313" s="11"/>
       <c r="C313" s="11"/>
       <c r="D313" s="11"/>
       <c r="E313" s="11"/>
     </row>
     <row r="314" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A314" s="18"/>
       <c r="B314" s="11"/>
       <c r="C314" s="11"/>
       <c r="D314" s="11"/>
       <c r="E314" s="11"/>
     </row>
     <row r="315" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A315" s="18"/>
       <c r="B315" s="11"/>
       <c r="C315" s="11"/>
       <c r="D315" s="11"/>
       <c r="E315" s="11"/>
     </row>
     <row r="316" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A316" s="18"/>
       <c r="B316" s="11"/>
       <c r="C316" s="11"/>
       <c r="D316" s="11"/>
       <c r="E316" s="11"/>
     </row>
     <row r="317" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A317" s="18"/>
       <c r="B317" s="11"/>
       <c r="C317" s="11"/>
       <c r="D317" s="11"/>
       <c r="E317" s="11"/>
     </row>
     <row r="318" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A318" s="18"/>
       <c r="B318" s="11"/>
       <c r="C318" s="11"/>
       <c r="D318" s="11"/>
       <c r="E318" s="11"/>
     </row>
     <row r="319" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A319" s="18"/>
       <c r="B319" s="11"/>
       <c r="C319" s="11"/>
       <c r="D319" s="11"/>
       <c r="E319" s="11"/>
     </row>
     <row r="320" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A320" s="18"/>
       <c r="B320" s="11"/>
       <c r="C320" s="11"/>
       <c r="D320" s="11"/>
       <c r="E320" s="11"/>
     </row>
     <row r="321" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A321" s="18"/>
       <c r="B321" s="11"/>
       <c r="C321" s="11"/>
       <c r="D321" s="11"/>
       <c r="E321" s="11"/>
     </row>
     <row r="322" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A322" s="18"/>
       <c r="B322" s="11"/>
       <c r="C322" s="11"/>
       <c r="D322" s="11"/>
       <c r="E322" s="11"/>
     </row>
     <row r="323" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A323" s="18"/>
       <c r="B323" s="11"/>
       <c r="C323" s="11"/>
       <c r="D323" s="11"/>
       <c r="E323" s="11"/>
     </row>
     <row r="324" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A324" s="18"/>
       <c r="B324" s="11"/>
       <c r="C324" s="11"/>
       <c r="D324" s="11"/>
       <c r="E324" s="11"/>
     </row>
     <row r="325" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A325" s="18"/>
       <c r="B325" s="11"/>
       <c r="C325" s="11"/>
       <c r="D325" s="11"/>
       <c r="E325" s="11"/>
     </row>
     <row r="326" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A326" s="18"/>
       <c r="B326" s="11"/>
       <c r="C326" s="11"/>
       <c r="D326" s="11"/>
       <c r="E326" s="11"/>
     </row>
     <row r="327" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A327" s="18"/>
       <c r="B327" s="11"/>
       <c r="C327" s="11"/>
       <c r="D327" s="11"/>
       <c r="E327" s="11"/>
     </row>
     <row r="328" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A328" s="18"/>
       <c r="B328" s="11"/>
       <c r="C328" s="11"/>
       <c r="D328" s="11"/>
       <c r="E328" s="11"/>
     </row>
     <row r="329" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A329" s="18"/>
       <c r="B329" s="11"/>
       <c r="C329" s="11"/>
       <c r="D329" s="11"/>
       <c r="E329" s="11"/>
     </row>
     <row r="330" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A330" s="18"/>
       <c r="B330" s="11"/>
       <c r="C330" s="11"/>
       <c r="D330" s="11"/>
       <c r="E330" s="11"/>
     </row>
     <row r="331" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A331" s="18"/>
       <c r="B331" s="11"/>
       <c r="C331" s="11"/>
       <c r="D331" s="11"/>
       <c r="E331" s="11"/>
     </row>
     <row r="332" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A332" s="18"/>
       <c r="B332" s="11"/>
       <c r="C332" s="11"/>
       <c r="D332" s="11"/>
       <c r="E332" s="11"/>
     </row>
     <row r="333" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A333" s="18"/>
       <c r="B333" s="11"/>
       <c r="C333" s="11"/>
       <c r="D333" s="11"/>
       <c r="E333" s="11"/>
     </row>
     <row r="334" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A334" s="18"/>
       <c r="B334" s="11"/>
       <c r="C334" s="11"/>
       <c r="D334" s="11"/>
       <c r="E334" s="11"/>
     </row>
     <row r="335" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A335" s="18"/>
       <c r="B335" s="11"/>
       <c r="C335" s="11"/>
       <c r="D335" s="11"/>
       <c r="E335" s="11"/>
     </row>
     <row r="336" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A336" s="18"/>
       <c r="B336" s="11"/>
       <c r="C336" s="11"/>
       <c r="D336" s="11"/>
       <c r="E336" s="11"/>
     </row>
     <row r="337" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A337" s="18"/>
       <c r="B337" s="11"/>
       <c r="C337" s="11"/>
       <c r="D337" s="11"/>
       <c r="E337" s="11"/>
     </row>
     <row r="338" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A338" s="18"/>
       <c r="B338" s="11"/>
       <c r="C338" s="11"/>
       <c r="D338" s="11"/>
       <c r="E338" s="11"/>
     </row>
     <row r="339" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A339" s="18"/>
       <c r="B339" s="11"/>
       <c r="C339" s="11"/>
       <c r="D339" s="11"/>
       <c r="E339" s="11"/>
     </row>
     <row r="340" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A340" s="18"/>
       <c r="B340" s="11"/>
       <c r="C340" s="11"/>
       <c r="D340" s="11"/>
       <c r="E340" s="11"/>
     </row>
     <row r="341" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A341" s="18"/>
       <c r="B341" s="11"/>
       <c r="C341" s="11"/>
       <c r="D341" s="11"/>
       <c r="E341" s="11"/>
     </row>
     <row r="342" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A342" s="18"/>
       <c r="B342" s="11"/>
       <c r="C342" s="11"/>
       <c r="D342" s="11"/>
       <c r="E342" s="11"/>
     </row>
     <row r="343" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A343" s="18"/>
       <c r="B343" s="11"/>
       <c r="C343" s="11"/>
       <c r="D343" s="11"/>
       <c r="E343" s="11"/>
     </row>
     <row r="344" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A344" s="18"/>
       <c r="B344" s="11"/>
       <c r="C344" s="11"/>
       <c r="D344" s="11"/>
       <c r="E344" s="11"/>
     </row>
     <row r="345" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A345" s="18"/>
       <c r="B345" s="11"/>
       <c r="C345" s="11"/>
       <c r="D345" s="11"/>
       <c r="E345" s="11"/>
     </row>
     <row r="346" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A346" s="18"/>
       <c r="B346" s="11"/>
       <c r="C346" s="11"/>
       <c r="D346" s="11"/>
       <c r="E346" s="11"/>
     </row>
     <row r="347" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A347" s="18"/>
       <c r="B347" s="11"/>
       <c r="C347" s="11"/>
       <c r="D347" s="11"/>
       <c r="E347" s="11"/>
     </row>
     <row r="348" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A348" s="18"/>
       <c r="B348" s="11"/>
       <c r="C348" s="11"/>
       <c r="D348" s="11"/>
       <c r="E348" s="11"/>
     </row>
     <row r="349" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A349" s="18"/>
       <c r="B349" s="11"/>
       <c r="C349" s="11"/>
       <c r="D349" s="11"/>
       <c r="E349" s="11"/>
     </row>
     <row r="350" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A350" s="18"/>
       <c r="B350" s="11"/>
       <c r="C350" s="11"/>
       <c r="D350" s="11"/>
       <c r="E350" s="11"/>
     </row>
     <row r="351" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A351" s="18"/>
       <c r="B351" s="11"/>
       <c r="C351" s="11"/>
       <c r="D351" s="11"/>
       <c r="E351" s="11"/>
     </row>
     <row r="352" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A352" s="18"/>
       <c r="B352" s="11"/>
       <c r="C352" s="11"/>
       <c r="D352" s="11"/>
       <c r="E352" s="11"/>
     </row>
     <row r="353" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A353" s="18"/>
       <c r="B353" s="11"/>
       <c r="C353" s="11"/>
       <c r="D353" s="11"/>
       <c r="E353" s="11"/>
     </row>
     <row r="354" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A354" s="18"/>
       <c r="B354" s="11"/>
       <c r="C354" s="11"/>
       <c r="D354" s="11"/>
       <c r="E354" s="11"/>
     </row>
     <row r="355" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A355" s="18"/>
       <c r="B355" s="11"/>
       <c r="C355" s="11"/>
       <c r="D355" s="11"/>
       <c r="E355" s="11"/>
     </row>
     <row r="356" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A356" s="18"/>
       <c r="B356" s="11"/>
       <c r="C356" s="11"/>
       <c r="D356" s="11"/>
       <c r="E356" s="11"/>
     </row>
     <row r="357" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A357" s="18"/>
       <c r="B357" s="11"/>
       <c r="C357" s="11"/>
       <c r="D357" s="11"/>
       <c r="E357" s="11"/>
     </row>
     <row r="358" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A358" s="18"/>
       <c r="B358" s="11"/>
       <c r="C358" s="11"/>
       <c r="D358" s="11"/>
       <c r="E358" s="11"/>
     </row>
     <row r="359" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A359" s="18"/>
       <c r="B359" s="11"/>
       <c r="C359" s="11"/>
       <c r="D359" s="11"/>

</xml_diff>

<commit_message>
update post-go-live trackers for 21-8940 and  21-4140
</commit_message>
<xml_diff>
--- a/teams/benefits-portfolio/benefits-intake-optimization-pingwind/post-go-live/21-4140/21-4140-post-go-live-submission-tracker.xlsx
+++ b/teams/benefits-portfolio/benefits-intake-optimization-pingwind/post-go-live/21-4140/21-4140-post-go-live-submission-tracker.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="212">
   <si>
     <t xml:space="preserve">21-4140 Post-Go-Live Submission Tracker</t>
   </si>
@@ -220,22 +220,37 @@
     <t xml:space="preserve">03/12/2026 10:46</t>
   </si>
   <si>
+    <t xml:space="preserve">Complete </t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/12/2026 13:13</t>
+  </si>
+  <si>
     <t xml:space="preserve">fc528242-5eca-499a-af53-08bbef6d190b</t>
   </si>
   <si>
     <t xml:space="preserve">03/12/2026 10:52</t>
   </si>
   <si>
+    <t xml:space="preserve">03/12/2026 13:15</t>
+  </si>
+  <si>
     <t xml:space="preserve">c69aa806-f001-4c11-8410-d92703eabfb1</t>
   </si>
   <si>
     <t xml:space="preserve">03/12/2026 19:11</t>
   </si>
   <si>
+    <t xml:space="preserve">03/12/2026 23:23</t>
+  </si>
+  <si>
     <t xml:space="preserve">5da48501-f708-4dcb-835c-6e0bda4aa140</t>
   </si>
   <si>
-    <t xml:space="preserve">03/13/2026 09:30</t>
+    <t xml:space="preserve">03/13/2026 9:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/13/2026 11:47</t>
   </si>
   <si>
     <t xml:space="preserve">c23fb21f-3ae9-49f4-baa8-73b544916ca8</t>
@@ -244,70 +259,106 @@
     <t xml:space="preserve">03/15/2026 21:10</t>
   </si>
   <si>
+    <t xml:space="preserve">03/16/2026 11:05</t>
+  </si>
+  <si>
     <t xml:space="preserve">563f9b82-d493-4b75-9ca6-cbd7cde54cb4</t>
   </si>
   <si>
     <t xml:space="preserve">03/16/2026 17:09</t>
   </si>
   <si>
+    <t xml:space="preserve">03/16/2026 19:35</t>
+  </si>
+  <si>
     <t xml:space="preserve">af362230-1f14-47b4-99bd-aef6bfaf0908</t>
   </si>
   <si>
     <t xml:space="preserve">03/16/2026 17:11</t>
   </si>
   <si>
+    <t xml:space="preserve">03/16/2026 19:32</t>
+  </si>
+  <si>
     <t xml:space="preserve">31958767-b377-4e47-bce5-582ce4e0daf9</t>
   </si>
   <si>
     <t xml:space="preserve">03/16/2026 20:26</t>
   </si>
   <si>
+    <t xml:space="preserve">03/17/2026 8:47</t>
+  </si>
+  <si>
     <t xml:space="preserve">80429ad7-605b-44e1-9c3c-e4476c93cf7f</t>
   </si>
   <si>
     <t xml:space="preserve">03/18/2026 13:32</t>
   </si>
   <si>
+    <t xml:space="preserve">03/18/2026 16:45</t>
+  </si>
+  <si>
     <t xml:space="preserve">e6297774-131c-4fad-beae-42bc1f763208</t>
   </si>
   <si>
     <t xml:space="preserve">03/18/2026 13:37</t>
   </si>
   <si>
+    <t xml:space="preserve">03/18/2026 16:43</t>
+  </si>
+  <si>
     <t xml:space="preserve">26054207-5940-4658-a4c6-f5905ed60f1d</t>
   </si>
   <si>
     <t xml:space="preserve">03/18/2026 14:50</t>
   </si>
   <si>
+    <t xml:space="preserve">03/18/2026 19:07</t>
+  </si>
+  <si>
     <t xml:space="preserve">6937e0ff-11ce-4871-8e1f-fea0481abc8e</t>
   </si>
   <si>
     <t xml:space="preserve">03/18/2026 15:09</t>
   </si>
   <si>
+    <t xml:space="preserve">03/18/2026 18:43</t>
+  </si>
+  <si>
     <t xml:space="preserve">7d27d9ba-40df-449e-b648-9ca84bd2e5ad</t>
   </si>
   <si>
     <t xml:space="preserve">03/19/2026 22:32</t>
   </si>
   <si>
+    <t xml:space="preserve">03/20/2026 9:08</t>
+  </si>
+  <si>
     <t xml:space="preserve">9a007d47-e752-41c3-858e-3e0f3a25d2a4</t>
   </si>
   <si>
     <t xml:space="preserve">03/20/2026 12:32</t>
   </si>
   <si>
+    <t xml:space="preserve">03/20/2026 14:11</t>
+  </si>
+  <si>
     <t xml:space="preserve">15ea917a-cca9-414d-a7e5-06945b40c68c</t>
   </si>
   <si>
     <t xml:space="preserve">03/20/2026 20:55</t>
   </si>
   <si>
+    <t xml:space="preserve">03/21/2026 9:52</t>
+  </si>
+  <si>
     <t xml:space="preserve">5d2df05b-36fb-44e8-8195-fadd2c48b859</t>
   </si>
   <si>
-    <t xml:space="preserve">03/23/2026 07:37</t>
+    <t xml:space="preserve">03/23/2026 7:37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/23/2026 9:54</t>
   </si>
   <si>
     <t xml:space="preserve">bf2c4d11-bfd6-431e-9fa1-9cc81e4ffe5f</t>
@@ -316,10 +367,16 @@
     <t xml:space="preserve">03/23/2026 10:59</t>
   </si>
   <si>
+    <t xml:space="preserve">03/23/2026 12:42</t>
+  </si>
+  <si>
     <t xml:space="preserve">d829f8ad-055b-4dca-a5e8-3aac12a01ff8</t>
   </si>
   <si>
-    <t xml:space="preserve">03/24/2026 01:14</t>
+    <t xml:space="preserve">03/24/2026 1:14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/24/2026 8:50</t>
   </si>
   <si>
     <t xml:space="preserve">3d7a0d9b-4743-4af3-9a92-50b82e9837a9</t>
@@ -328,10 +385,16 @@
     <t xml:space="preserve">03/24/2026 14:14</t>
   </si>
   <si>
+    <t xml:space="preserve">03/24/2026 17:53</t>
+  </si>
+  <si>
     <t xml:space="preserve">fb54d4a6-e6b4-4818-aae2-04e99dccf8ce</t>
   </si>
   <si>
-    <t xml:space="preserve">03/25/2026 08:27</t>
+    <t xml:space="preserve">03/25/2026 8:27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/25/2026 10:27</t>
   </si>
   <si>
     <t xml:space="preserve">8d929786-87d7-4351-818c-482fdb0559f2</t>
@@ -340,40 +403,61 @@
     <t xml:space="preserve">03/25/2026 10:24</t>
   </si>
   <si>
+    <t xml:space="preserve">03/25/2026 12:07</t>
+  </si>
+  <si>
     <t xml:space="preserve">a727ea0c-f323-435d-8700-9e2bddba8fb6</t>
   </si>
   <si>
     <t xml:space="preserve">03/26/2026 13:50</t>
   </si>
   <si>
+    <t xml:space="preserve">03/26/2026 15:58</t>
+  </si>
+  <si>
     <t xml:space="preserve">3a8b5ee6-c30e-4622-9ca9-248f78d20546</t>
   </si>
   <si>
     <t xml:space="preserve">03/26/2026 18:45</t>
   </si>
   <si>
+    <t xml:space="preserve">03/27/2026 7:46</t>
+  </si>
+  <si>
     <t xml:space="preserve">d35c90c0-489e-4873-abce-c85961170979</t>
   </si>
   <si>
     <t xml:space="preserve">03/26/2026 19:37</t>
   </si>
   <si>
+    <t xml:space="preserve">03/27/2026 8:41</t>
+  </si>
+  <si>
     <t xml:space="preserve">90d8293d-915e-4db2-9872-b184853f0b39</t>
   </si>
   <si>
     <t xml:space="preserve">03/26/2026 20:15</t>
   </si>
   <si>
+    <t xml:space="preserve">03/27/2026 9:10</t>
+  </si>
+  <si>
     <t xml:space="preserve">2fe104bc-bc1b-4463-bbc5-0af5f49ba8f1</t>
   </si>
   <si>
     <t xml:space="preserve">03/26/2026 22:48</t>
   </si>
   <si>
+    <t xml:space="preserve">03/27/2026 10:00</t>
+  </si>
+  <si>
     <t xml:space="preserve">24b3ebc7-489a-4451-b5af-02fa595cc584</t>
   </si>
   <si>
-    <t xml:space="preserve">03/27/2026 08:54</t>
+    <t xml:space="preserve">03/27/2026 8:54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/27/2026 11:03</t>
   </si>
   <si>
     <t xml:space="preserve">b9d11296-72fb-4fc4-80eb-b8e6885773ed</t>
@@ -382,16 +466,25 @@
     <t xml:space="preserve">03/27/2026 14:34</t>
   </si>
   <si>
+    <t xml:space="preserve">03/27/2026 16:48</t>
+  </si>
+  <si>
     <t xml:space="preserve">704b5e6a-1953-4c74-bd6d-392e0f5093f6</t>
   </si>
   <si>
     <t xml:space="preserve">03/27/2026 19:10</t>
   </si>
   <si>
+    <t xml:space="preserve">03/28/2026 8:47</t>
+  </si>
+  <si>
     <t xml:space="preserve">26a4f23d-94b9-4194-b864-aa884a027574</t>
   </si>
   <si>
-    <t xml:space="preserve">03/28/2026 01:53</t>
+    <t xml:space="preserve">03/28/2026 1:53</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/28/2026 11:02</t>
   </si>
   <si>
     <t xml:space="preserve">5e22bf60-b82f-47bc-92a4-091d556d9dd5</t>
@@ -400,16 +493,25 @@
     <t xml:space="preserve">03/28/2026 10:49</t>
   </si>
   <si>
+    <t xml:space="preserve">03/28/2026 11:39</t>
+  </si>
+  <si>
     <t xml:space="preserve">d2e4adab-bbde-4d68-9320-f60c5072c194</t>
   </si>
   <si>
     <t xml:space="preserve">03/28/2026 20:28</t>
   </si>
   <si>
+    <t xml:space="preserve">03/30/2026 8:43</t>
+  </si>
+  <si>
     <t xml:space="preserve">a95d817f-80bc-4d76-bad7-714adf8f9b93</t>
   </si>
   <si>
-    <t xml:space="preserve">03/29/2026 06:57</t>
+    <t xml:space="preserve">03/29/2026 6:57</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/30/2026 8:58</t>
   </si>
   <si>
     <t xml:space="preserve">6ff9696e-4b29-462e-99f6-d0373143e945</t>
@@ -418,10 +520,16 @@
     <t xml:space="preserve">03/29/2026 18:15</t>
   </si>
   <si>
+    <t xml:space="preserve">03/30/2026 11:58</t>
+  </si>
+  <si>
     <t xml:space="preserve">5591c8cf-0399-44a9-8efa-2bd9536b97c2</t>
   </si>
   <si>
-    <t xml:space="preserve">03/30/2026 05:20</t>
+    <t xml:space="preserve">03/30/2026 5:20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/30/2026 10:51</t>
   </si>
   <si>
     <t xml:space="preserve">76bebd21-5dfe-44b3-99ce-6ffcceb6ccb8</t>
@@ -430,34 +538,52 @@
     <t xml:space="preserve">03/30/2026 10:42</t>
   </si>
   <si>
+    <t xml:space="preserve">03/30/2026 13:28</t>
+  </si>
+  <si>
     <t xml:space="preserve">2570e4df-7a2b-4677-be74-2895137445c0</t>
   </si>
   <si>
     <t xml:space="preserve">03/30/2026 11:00</t>
   </si>
   <si>
+    <t xml:space="preserve">03/30/2026 13:55</t>
+  </si>
+  <si>
     <t xml:space="preserve">589b3dc5-f296-448a-9430-ab48d0428913</t>
   </si>
   <si>
     <t xml:space="preserve">03/30/2026 12:18</t>
   </si>
   <si>
+    <t xml:space="preserve">03/30/2026 15:50</t>
+  </si>
+  <si>
     <t xml:space="preserve">b6570d1a-4401-47e5-9387-b78e44c992c9</t>
   </si>
   <si>
     <t xml:space="preserve">03/30/2026 18:44</t>
   </si>
   <si>
+    <t xml:space="preserve">03/31/2026 0:17</t>
+  </si>
+  <si>
     <t xml:space="preserve">aa1d974b-9e45-44fb-8b85-9905b25b44c3</t>
   </si>
   <si>
     <t xml:space="preserve">03/30/2026 21:18</t>
   </si>
   <si>
+    <t xml:space="preserve">03/31/2026 8:20</t>
+  </si>
+  <si>
     <t xml:space="preserve">697e2deb-3207-4444-99e8-5f8d52baf28a</t>
   </si>
   <si>
-    <t xml:space="preserve">03/31/2026 07:47</t>
+    <t xml:space="preserve">03/31/2026 7:47</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/31/2026 10:08</t>
   </si>
   <si>
     <t xml:space="preserve">89968a27-b320-4c65-93fe-293aa3e851b9</t>
@@ -466,16 +592,25 @@
     <t xml:space="preserve">03/31/2026 14:05</t>
   </si>
   <si>
+    <t xml:space="preserve">03/31/2026 17:39</t>
+  </si>
+  <si>
     <t xml:space="preserve">6f7274a2-5a07-49b4-aca6-86c98edd8c53</t>
   </si>
   <si>
     <t xml:space="preserve">03/31/2026 16:02</t>
   </si>
   <si>
+    <t xml:space="preserve">03/31/2026 18:21</t>
+  </si>
+  <si>
     <t xml:space="preserve">5425c3b4-c4d2-417d-84d3-e99cefdcdeb3</t>
   </si>
   <si>
-    <t xml:space="preserve">04/01/2026 09:48</t>
+    <t xml:space="preserve">04/01/2026 9:48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04/01/2026 11:43</t>
   </si>
   <si>
     <t xml:space="preserve">9121103f-ef2e-4fcf-a827-e28ca388c475</t>
@@ -484,16 +619,25 @@
     <t xml:space="preserve">04/02/2026 17:34</t>
   </si>
   <si>
+    <t xml:space="preserve">04/02/2026 21:21</t>
+  </si>
+  <si>
     <t xml:space="preserve">2ec7c563-a71d-4f6d-81f2-a2bd930be182</t>
   </si>
   <si>
     <t xml:space="preserve">04/03/2026 14:02</t>
   </si>
   <si>
+    <t xml:space="preserve">04/03/2026 16:24</t>
+  </si>
+  <si>
     <t xml:space="preserve">327f7b82-2265-4fe8-b774-fd092b52f9b9</t>
   </si>
   <si>
-    <t xml:space="preserve">04/04/2026 05:07</t>
+    <t xml:space="preserve">04/04/2026 5:07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04/04/2026 14:07</t>
   </si>
   <si>
     <t xml:space="preserve">49b389bc-cef5-4979-b4f1-7ef98b6c38a2</t>
@@ -502,10 +646,16 @@
     <t xml:space="preserve">04/05/2026 12:22</t>
   </si>
   <si>
+    <t xml:space="preserve">04/06/2026 8:32</t>
+  </si>
+  <si>
     <t xml:space="preserve">e1132c43-a626-4f78-a569-69615fd10b54</t>
   </si>
   <si>
     <t xml:space="preserve">04/05/2026 23:05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04/06/2026 9:27</t>
   </si>
 </sst>
 </file>
@@ -1832,8 +1982,15 @@
       <c r="C52" s="13" t="n">
         <v>46090.8319444444</v>
       </c>
-      <c r="D52" s="11"/>
-      <c r="E52" s="13"/>
+      <c r="D52" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E52" s="13" t="n">
+        <v>46091.3465277778</v>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>69756221</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="10" t="s">
@@ -1845,8 +2002,15 @@
       <c r="C53" s="13" t="n">
         <v>46090.9305555556</v>
       </c>
-      <c r="D53" s="11"/>
-      <c r="E53" s="13"/>
+      <c r="D53" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E53" s="13" t="n">
+        <v>46091.3930555556</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>69758255</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="10" t="s">
@@ -1858,8 +2022,15 @@
       <c r="C54" s="13" t="n">
         <v>46091.4236111111</v>
       </c>
-      <c r="D54" s="11"/>
-      <c r="E54" s="13"/>
+      <c r="D54" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E54" s="13" t="n">
+        <v>46091.5819444444</v>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>69766917</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="10" t="s">
@@ -1871,632 +2042,975 @@
       <c r="C55" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="D55" s="11"/>
-      <c r="E55" s="13"/>
+      <c r="D55" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E55" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>69857804</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="10" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B56" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C56" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="D56" s="11"/>
-      <c r="E56" s="13"/>
+        <v>69</v>
+      </c>
+      <c r="D56" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E56" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>69858466</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="10" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B57" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C57" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="D57" s="11"/>
-      <c r="E57" s="13"/>
+        <v>72</v>
+      </c>
+      <c r="D57" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E57" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="F57" s="2" t="n">
+        <v>69891093</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B58" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="D58" s="11"/>
-      <c r="E58" s="13"/>
+        <v>75</v>
+      </c>
+      <c r="D58" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E58" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="F58" s="2" t="n">
+        <v>69899372</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="10" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B59" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C59" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="D59" s="11"/>
-      <c r="E59" s="13"/>
+        <v>78</v>
+      </c>
+      <c r="D59" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E59" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>69951836</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="10" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="B60" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="D60" s="11"/>
-      <c r="E60" s="13"/>
+        <v>81</v>
+      </c>
+      <c r="D60" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E60" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>69983511</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="10" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B61" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C61" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="D61" s="11"/>
-      <c r="E61" s="13"/>
+        <v>84</v>
+      </c>
+      <c r="D61" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E61" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="F61" s="2" t="n">
+        <v>69983999</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="10" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="B62" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C62" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="D62" s="11"/>
-      <c r="E62" s="13"/>
+        <v>87</v>
+      </c>
+      <c r="D62" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E62" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>69989082</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="10" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="B63" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C63" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="D63" s="11"/>
-      <c r="E63" s="13"/>
+        <v>90</v>
+      </c>
+      <c r="D63" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E63" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="F63" s="2" t="n">
+        <v>70062700</v>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="10" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="B64" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C64" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="D64" s="11"/>
-      <c r="E64" s="13"/>
+        <v>93</v>
+      </c>
+      <c r="D64" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E64" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>70062899</v>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="10" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="B65" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C65" s="13" t="s">
-        <v>85</v>
-      </c>
-      <c r="D65" s="11"/>
-      <c r="E65" s="13"/>
+        <v>96</v>
+      </c>
+      <c r="D65" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E65" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="F65" s="2" t="n">
+        <v>70067180</v>
+      </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="10" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="B66" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C66" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="D66" s="11"/>
-      <c r="E66" s="13"/>
+        <v>99</v>
+      </c>
+      <c r="D66" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E66" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>70068382</v>
+      </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="10" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="B67" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C67" s="13" t="s">
-        <v>89</v>
-      </c>
-      <c r="D67" s="11"/>
-      <c r="E67" s="13"/>
+        <v>102</v>
+      </c>
+      <c r="D67" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E67" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="F67" s="2" t="n">
+        <v>70127222</v>
+      </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="18" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="B68" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C68" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="D68" s="11"/>
-      <c r="E68" s="13"/>
+        <v>105</v>
+      </c>
+      <c r="D68" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E68" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>70146390</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="18" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="B69" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C69" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="D69" s="11"/>
-      <c r="E69" s="13"/>
+        <v>108</v>
+      </c>
+      <c r="D69" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E69" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>70166234</v>
+      </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="18" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="B70" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C70" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="D70" s="11"/>
-      <c r="E70" s="13"/>
+        <v>111</v>
+      </c>
+      <c r="D70" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E70" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="F70" s="2" t="n">
+        <v>70185588</v>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="18" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="B71" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C71" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="D71" s="11"/>
-      <c r="E71" s="11"/>
+        <v>114</v>
+      </c>
+      <c r="D71" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E71" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="F71" s="2" t="n">
+        <v>70194624</v>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="18" t="s">
-        <v>98</v>
+        <v>116</v>
       </c>
       <c r="B72" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C72" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="D72" s="11"/>
-      <c r="E72" s="11"/>
+        <v>117</v>
+      </c>
+      <c r="D72" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E72" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="F72" s="2" t="n">
+        <v>70238236</v>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="18" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="B73" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C73" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="D73" s="11"/>
-      <c r="E73" s="11"/>
+        <v>120</v>
+      </c>
+      <c r="D73" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E73" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="F73" s="2" t="n">
+        <v>70266016</v>
+      </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="18" t="s">
-        <v>102</v>
+        <v>122</v>
       </c>
       <c r="B74" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C74" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="D74" s="11"/>
-      <c r="E74" s="11"/>
+        <v>123</v>
+      </c>
+      <c r="D74" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E74" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="F74" s="2" t="n">
+        <v>70286404</v>
+      </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="18" t="s">
-        <v>104</v>
+        <v>125</v>
       </c>
       <c r="B75" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C75" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="D75" s="11"/>
-      <c r="E75" s="11"/>
+        <v>126</v>
+      </c>
+      <c r="D75" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E75" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="F75" s="2" t="n">
+        <v>70291283</v>
+      </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="18" t="s">
-        <v>106</v>
+        <v>128</v>
       </c>
       <c r="B76" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C76" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="D76" s="11"/>
-      <c r="E76" s="11"/>
+        <v>129</v>
+      </c>
+      <c r="D76" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E76" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>70347261</v>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="18" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="B77" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C77" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="D77" s="11"/>
-      <c r="E77" s="11"/>
+        <v>132</v>
+      </c>
+      <c r="D77" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E77" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="F77" s="2" t="n">
+        <v>70362729</v>
+      </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="18" t="s">
-        <v>110</v>
+        <v>134</v>
       </c>
       <c r="B78" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C78" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="D78" s="11"/>
-      <c r="E78" s="11"/>
+        <v>135</v>
+      </c>
+      <c r="D78" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E78" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="F78" s="2" t="n">
+        <v>70363889</v>
+      </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="18" t="s">
-        <v>112</v>
+        <v>137</v>
       </c>
       <c r="B79" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C79" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="D79" s="11"/>
-      <c r="E79" s="11"/>
+        <v>138</v>
+      </c>
+      <c r="D79" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E79" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="F79" s="2" t="n">
+        <v>70364488</v>
+      </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="18" t="s">
-        <v>114</v>
+        <v>140</v>
       </c>
       <c r="B80" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C80" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="D80" s="11"/>
-      <c r="E80" s="11"/>
+        <v>141</v>
+      </c>
+      <c r="D80" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E80" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="F80" s="2" t="n">
+        <v>70366249</v>
+      </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="18" t="s">
-        <v>116</v>
+        <v>143</v>
       </c>
       <c r="B81" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C81" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="D81" s="11"/>
-      <c r="E81" s="11"/>
+        <v>144</v>
+      </c>
+      <c r="D81" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E81" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="F81" s="2" t="n">
+        <v>70369157</v>
+      </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="18" t="s">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="B82" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C82" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="D82" s="11"/>
-      <c r="E82" s="11"/>
+        <v>147</v>
+      </c>
+      <c r="D82" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E82" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="F82" s="2" t="n">
+        <v>70392574</v>
+      </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="18" t="s">
-        <v>120</v>
+        <v>149</v>
       </c>
       <c r="B83" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C83" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="D83" s="11"/>
-      <c r="E83" s="11"/>
+        <v>150</v>
+      </c>
+      <c r="D83" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E83" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="F83" s="2" t="n">
+        <v>70403708</v>
+      </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="18" t="s">
-        <v>122</v>
+        <v>152</v>
       </c>
       <c r="B84" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C84" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="D84" s="11"/>
-      <c r="E84" s="11"/>
+        <v>153</v>
+      </c>
+      <c r="D84" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E84" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="F84" s="2" t="n">
+        <v>70406817</v>
+      </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="18" t="s">
-        <v>124</v>
+        <v>155</v>
       </c>
       <c r="B85" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C85" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="D85" s="11"/>
-      <c r="E85" s="11"/>
+        <v>156</v>
+      </c>
+      <c r="D85" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E85" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="F85" s="2" t="n">
+        <v>70408173</v>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="18" t="s">
-        <v>126</v>
+        <v>158</v>
       </c>
       <c r="B86" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C86" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="D86" s="11"/>
-      <c r="E86" s="11"/>
+        <v>159</v>
+      </c>
+      <c r="D86" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E86" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="F86" s="2" t="n">
+        <v>70415578</v>
+      </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="18" t="s">
-        <v>128</v>
+        <v>161</v>
       </c>
       <c r="B87" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C87" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="D87" s="11"/>
-      <c r="E87" s="11"/>
+        <v>162</v>
+      </c>
+      <c r="D87" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E87" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="F87" s="2" t="n">
+        <v>70417353</v>
+      </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="18" t="s">
-        <v>130</v>
+        <v>164</v>
       </c>
       <c r="B88" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C88" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="D88" s="11"/>
-      <c r="E88" s="11"/>
+        <v>165</v>
+      </c>
+      <c r="D88" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E88" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="F88" s="2" t="n">
+        <v>70421663</v>
+      </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="18" t="s">
-        <v>132</v>
+        <v>167</v>
       </c>
       <c r="B89" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C89" s="11" t="s">
-        <v>133</v>
-      </c>
-      <c r="D89" s="11"/>
-      <c r="E89" s="11"/>
+        <v>168</v>
+      </c>
+      <c r="D89" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E89" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="F89" s="2" t="n">
+        <v>70424535</v>
+      </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="18" t="s">
-        <v>134</v>
+        <v>170</v>
       </c>
       <c r="B90" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C90" s="11" t="s">
-        <v>135</v>
-      </c>
-      <c r="D90" s="11"/>
-      <c r="E90" s="11"/>
+        <v>171</v>
+      </c>
+      <c r="D90" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E90" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="F90" s="2" t="n">
+        <v>70432150</v>
+      </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="18" t="s">
-        <v>136</v>
+        <v>173</v>
       </c>
       <c r="B91" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C91" s="11" t="s">
-        <v>137</v>
-      </c>
-      <c r="D91" s="11"/>
-      <c r="E91" s="11"/>
+        <v>174</v>
+      </c>
+      <c r="D91" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E91" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="F91" s="2" t="n">
+        <v>70435337</v>
+      </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="18" t="s">
-        <v>138</v>
+        <v>176</v>
       </c>
       <c r="B92" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C92" s="11" t="s">
-        <v>139</v>
-      </c>
-      <c r="D92" s="11"/>
-      <c r="E92" s="11"/>
+        <v>177</v>
+      </c>
+      <c r="D92" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E92" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="F92" s="2" t="n">
+        <v>70442379</v>
+      </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="18" t="s">
-        <v>140</v>
+        <v>179</v>
       </c>
       <c r="B93" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C93" s="11" t="s">
-        <v>141</v>
-      </c>
-      <c r="D93" s="11"/>
-      <c r="E93" s="11"/>
+        <v>180</v>
+      </c>
+      <c r="D93" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E93" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="F93" s="2" t="n">
+        <v>70471341</v>
+      </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="18" t="s">
-        <v>142</v>
+        <v>182</v>
       </c>
       <c r="B94" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C94" s="11" t="s">
-        <v>143</v>
-      </c>
-      <c r="D94" s="11"/>
-      <c r="E94" s="11"/>
+        <v>183</v>
+      </c>
+      <c r="D94" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E94" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="F94" s="2" t="n">
+        <v>70473754</v>
+      </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="18" t="s">
-        <v>144</v>
+        <v>185</v>
       </c>
       <c r="B95" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C95" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="D95" s="11"/>
-      <c r="E95" s="11"/>
+        <v>186</v>
+      </c>
+      <c r="D95" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E95" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="F95" s="2" t="n">
+        <v>70477314</v>
+      </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="18" t="s">
-        <v>146</v>
+        <v>188</v>
       </c>
       <c r="B96" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C96" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="D96" s="11"/>
-      <c r="E96" s="11"/>
+        <v>189</v>
+      </c>
+      <c r="D96" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E96" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="F96" s="2" t="n">
+        <v>70501361</v>
+      </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="18" t="s">
-        <v>148</v>
+        <v>191</v>
       </c>
       <c r="B97" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C97" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="D97" s="11"/>
-      <c r="E97" s="11"/>
+        <v>192</v>
+      </c>
+      <c r="D97" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E97" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="F97" s="2" t="n">
+        <v>70508759</v>
+      </c>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="18" t="s">
-        <v>150</v>
+        <v>194</v>
       </c>
       <c r="B98" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C98" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="D98" s="11"/>
-      <c r="E98" s="11"/>
+        <v>195</v>
+      </c>
+      <c r="D98" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E98" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="F98" s="2" t="n">
+        <v>70525957</v>
+      </c>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="18" t="s">
-        <v>152</v>
+        <v>197</v>
       </c>
       <c r="B99" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C99" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="D99" s="11"/>
-      <c r="E99" s="11"/>
+        <v>198</v>
+      </c>
+      <c r="D99" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E99" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="F99" s="2" t="n">
+        <v>70597654</v>
+      </c>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="18" t="s">
-        <v>154</v>
+        <v>200</v>
       </c>
       <c r="B100" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C100" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="D100" s="11"/>
-      <c r="E100" s="11"/>
+        <v>201</v>
+      </c>
+      <c r="D100" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E100" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="F100" s="2" t="n">
+        <v>70624024</v>
+      </c>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="18" t="s">
-        <v>156</v>
+        <v>203</v>
       </c>
       <c r="B101" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C101" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="D101" s="11"/>
-      <c r="E101" s="11"/>
+        <v>204</v>
+      </c>
+      <c r="D101" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E101" s="11" t="s">
+        <v>205</v>
+      </c>
+      <c r="F101" s="2" t="n">
+        <v>70640675</v>
+      </c>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="18" t="s">
-        <v>158</v>
+        <v>206</v>
       </c>
       <c r="B102" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C102" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="D102" s="11"/>
-      <c r="E102" s="11"/>
+        <v>207</v>
+      </c>
+      <c r="D102" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E102" s="11" t="s">
+        <v>208</v>
+      </c>
+      <c r="F102" s="2" t="n">
+        <v>70648458</v>
+      </c>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="18" t="s">
-        <v>160</v>
+        <v>209</v>
       </c>
       <c r="B103" s="11" t="s">
         <v>64</v>
       </c>
       <c r="C103" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="D103" s="11"/>
-      <c r="E103" s="11"/>
+        <v>210</v>
+      </c>
+      <c r="D103" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E103" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="F103" s="2" t="n">
+        <v>70651247</v>
+      </c>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="18"/>

</xml_diff>